<commit_message>
fixing boxplots and spatial heatmaps
also added more ROIs to spreadsheet
</commit_message>
<xml_diff>
--- a/fake_data_for_testing.xlsx
+++ b/fake_data_for_testing.xlsx
@@ -5,17 +5,24 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Bryn\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AngelLab\Documents\GitHub\spatial-proteomics-analyzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B3D1240-5752-4D15-A321-9CC05D0C891B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08A553ED-EF7F-459B-95EC-920DA87AEA73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="1725" windowWidth="37710" windowHeight="19875" activeTab="1" xr2:uid="{F6399DF4-9833-403B-881F-8C907DE7D545}"/>
+    <workbookView xWindow="8550" yWindow="6720" windowWidth="31185" windowHeight="19875" activeTab="9" xr2:uid="{F6399DF4-9833-403B-881F-8C907DE7D545}"/>
   </bookViews>
   <sheets>
     <sheet name="ROI_101" sheetId="1" r:id="rId1"/>
     <sheet name="ROI_102" sheetId="2" r:id="rId2"/>
     <sheet name="ROI_103" sheetId="3" r:id="rId3"/>
+    <sheet name="ROI_104" sheetId="4" r:id="rId4"/>
+    <sheet name="ROI_105" sheetId="7" r:id="rId5"/>
+    <sheet name="ROI_106" sheetId="8" r:id="rId6"/>
+    <sheet name="ROI_107" sheetId="9" r:id="rId7"/>
+    <sheet name="ROI_108" sheetId="10" r:id="rId8"/>
+    <sheet name="ROI_109" sheetId="5" r:id="rId9"/>
+    <sheet name="ROI_110" sheetId="6" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="34">
   <si>
     <t>Spot index</t>
   </si>
@@ -78,6 +85,69 @@
   </si>
   <si>
     <t>Spot 23071</t>
+  </si>
+  <si>
+    <t>Spot 28469</t>
+  </si>
+  <si>
+    <t>Spot 28470</t>
+  </si>
+  <si>
+    <t>Spot 28471</t>
+  </si>
+  <si>
+    <t>Spot 34019</t>
+  </si>
+  <si>
+    <t>Spot 34020</t>
+  </si>
+  <si>
+    <t>Spot 34021</t>
+  </si>
+  <si>
+    <t>Spot 37474</t>
+  </si>
+  <si>
+    <t>Spot 37475</t>
+  </si>
+  <si>
+    <t>Spot 37476</t>
+  </si>
+  <si>
+    <t>Spot 43859</t>
+  </si>
+  <si>
+    <t>Spot 43860</t>
+  </si>
+  <si>
+    <t>Spot 43861</t>
+  </si>
+  <si>
+    <t>Spot 49334</t>
+  </si>
+  <si>
+    <t>Spot 49335</t>
+  </si>
+  <si>
+    <t>Spot 49336</t>
+  </si>
+  <si>
+    <t>Spot 54690</t>
+  </si>
+  <si>
+    <t>Spot 54691</t>
+  </si>
+  <si>
+    <t>Spot 54692</t>
+  </si>
+  <si>
+    <t>Spot 60019</t>
+  </si>
+  <si>
+    <t>Spot 60020</t>
+  </si>
+  <si>
+    <t>Spot 60021</t>
   </si>
 </sst>
 </file>
@@ -113,7 +183,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -532,6 +609,111 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB6282AF-55EE-452C-B389-599A7CE5298B}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10">
+        <v>758.45190000000002</v>
+      </c>
+      <c r="F1" s="10">
+        <v>797.42639999999994</v>
+      </c>
+      <c r="G1" s="10">
+        <v>976.45169999999996</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="10">
+        <v>60019</v>
+      </c>
+      <c r="B2" s="10">
+        <v>-33089.45703125</v>
+      </c>
+      <c r="C2" s="10">
+        <v>20646.685546875</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="10">
+        <v>256.15579525240003</v>
+      </c>
+      <c r="F2" s="10">
+        <v>955.68828809765</v>
+      </c>
+      <c r="G2" s="10">
+        <v>241.66380071978</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="10">
+        <v>60020</v>
+      </c>
+      <c r="B3" s="10">
+        <v>-33069.45703125</v>
+      </c>
+      <c r="C3" s="10">
+        <v>20646.685546875</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="10">
+        <v>265.42921170273002</v>
+      </c>
+      <c r="F3" s="10">
+        <v>1460.4402041286</v>
+      </c>
+      <c r="G3" s="10">
+        <v>581.27838283371</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="10">
+        <v>60021</v>
+      </c>
+      <c r="B4" s="10">
+        <v>-33049.45703125</v>
+      </c>
+      <c r="C4" s="10">
+        <v>20646.685546875</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="10">
+        <v>483.84765406101002</v>
+      </c>
+      <c r="F4" s="10">
+        <v>1211.4067496380001</v>
+      </c>
+      <c r="G4" s="10">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F296F55-5544-4735-AC2B-A3FA67987D68}">
   <dimension ref="A1:G4"/>
@@ -638,6 +820,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835AC33F-2B2E-495D-A0E2-411CB48665CE}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
@@ -734,4 +919,643 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFDEB40D-D7AE-49DA-ADE5-877F144CE992}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4">
+        <v>758.45190000000002</v>
+      </c>
+      <c r="F1" s="4">
+        <v>797.42639999999994</v>
+      </c>
+      <c r="G1" s="4">
+        <v>976.45169999999996</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>28469</v>
+      </c>
+      <c r="B2" s="4">
+        <v>-27490.068359375</v>
+      </c>
+      <c r="C2" s="4">
+        <v>32713.32421875</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="4">
+        <v>420.99027199733001</v>
+      </c>
+      <c r="F2" s="4">
+        <v>1211.9416921135</v>
+      </c>
+      <c r="G2" s="4">
+        <v>408.72365568038998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>28470</v>
+      </c>
+      <c r="B3" s="4">
+        <v>-27470.068359375</v>
+      </c>
+      <c r="C3" s="4">
+        <v>32713.32421875</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="4">
+        <v>446.7628716676</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1466.5041348013001</v>
+      </c>
+      <c r="G3" s="4">
+        <v>295.50459000435001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>28471</v>
+      </c>
+      <c r="B4" s="4">
+        <v>-27450.068359375</v>
+      </c>
+      <c r="C4" s="4">
+        <v>32713.32421875</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="4">
+        <v>490.93842046242003</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1169.4347458504001</v>
+      </c>
+      <c r="G4" s="4">
+        <v>340.74264799218003</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31ADDFC5-19D6-44D6-9C96-44266C0BC057}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="5">
+        <v>758.45190000000002</v>
+      </c>
+      <c r="F1" s="5">
+        <v>797.42639999999994</v>
+      </c>
+      <c r="G1" s="5">
+        <v>976.45169999999996</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="5">
+        <v>34019</v>
+      </c>
+      <c r="B2" s="5">
+        <v>-32746.869140625</v>
+      </c>
+      <c r="C2" s="5">
+        <v>32768.18359375</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="5">
+        <v>440.28731580162003</v>
+      </c>
+      <c r="F2" s="5">
+        <v>2237.2022153057001</v>
+      </c>
+      <c r="G2" s="5">
+        <v>559.91720272811006</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="5">
+        <v>34020</v>
+      </c>
+      <c r="B3" s="5">
+        <v>-32766.869140625</v>
+      </c>
+      <c r="C3" s="5">
+        <v>32748.181640625</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="5">
+        <v>332.29694807494002</v>
+      </c>
+      <c r="F3" s="5">
+        <v>2818.5901845642002</v>
+      </c>
+      <c r="G3" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>34021</v>
+      </c>
+      <c r="B4" s="5">
+        <v>-32746.869140625</v>
+      </c>
+      <c r="C4" s="5">
+        <v>32748.181640625</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="5">
+        <v>320.89495010078002</v>
+      </c>
+      <c r="F4" s="5">
+        <v>1438.2079369802</v>
+      </c>
+      <c r="G4" s="5">
+        <v>668.39259036534997</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0202B7-E9CB-4AD1-95D6-D6F5D7E09B30}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6">
+        <v>758.45190000000002</v>
+      </c>
+      <c r="F1" s="6">
+        <v>797.42639999999994</v>
+      </c>
+      <c r="G1" s="6">
+        <v>976.45169999999996</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
+        <v>37474</v>
+      </c>
+      <c r="B2" s="6">
+        <v>-30717.412109375</v>
+      </c>
+      <c r="C2" s="6">
+        <v>31830.18359375</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="6">
+        <v>520.47706409116995</v>
+      </c>
+      <c r="F2" s="6">
+        <v>1522.1108574118</v>
+      </c>
+      <c r="G2" s="6">
+        <v>588.77027727211998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>37475</v>
+      </c>
+      <c r="B3" s="6">
+        <v>-30697.412109375</v>
+      </c>
+      <c r="C3" s="6">
+        <v>31830.18359375</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="6">
+        <v>355.87143518788997</v>
+      </c>
+      <c r="F3" s="6">
+        <v>1393.2856418939</v>
+      </c>
+      <c r="G3" s="6">
+        <v>557.47750053515006</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>37476</v>
+      </c>
+      <c r="B4" s="6">
+        <v>-30677.412109375</v>
+      </c>
+      <c r="C4" s="6">
+        <v>31830.18359375</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="6">
+        <v>795.17653357029997</v>
+      </c>
+      <c r="F4" s="6">
+        <v>1712.9573784839999</v>
+      </c>
+      <c r="G4" s="6">
+        <v>405.17805748735998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A0A7254-37F6-48CA-B819-97367EFD6006}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="7">
+        <v>758.45190000000002</v>
+      </c>
+      <c r="F1" s="7">
+        <v>797.42639999999994</v>
+      </c>
+      <c r="G1" s="7">
+        <v>976.45169999999996</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>43859</v>
+      </c>
+      <c r="B2" s="7">
+        <v>-33603.2109375</v>
+      </c>
+      <c r="C2" s="7">
+        <v>28940.3359375</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="7">
+        <v>291.09056336352</v>
+      </c>
+      <c r="F2" s="7">
+        <v>436.54272586313999</v>
+      </c>
+      <c r="G2" s="7">
+        <v>139.30629647851001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>43860</v>
+      </c>
+      <c r="B3" s="7">
+        <v>-33583.2109375</v>
+      </c>
+      <c r="C3" s="7">
+        <v>28940.3359375</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="7">
+        <v>353.94345738353002</v>
+      </c>
+      <c r="F3" s="7">
+        <v>452.18327511971</v>
+      </c>
+      <c r="G3" s="7">
+        <v>75.830735075384993</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>43861</v>
+      </c>
+      <c r="B4" s="7">
+        <v>-33563.2109375</v>
+      </c>
+      <c r="C4" s="7">
+        <v>28940.3359375</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="7">
+        <v>397.93196587118001</v>
+      </c>
+      <c r="F4" s="7">
+        <v>758.09788334146003</v>
+      </c>
+      <c r="G4" s="7">
+        <v>95.525887131671993</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31F6CDFB-E1F5-460A-8FBB-26E642781AAA}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="8">
+        <v>758.45190000000002</v>
+      </c>
+      <c r="F1" s="8">
+        <v>797.42639999999994</v>
+      </c>
+      <c r="G1" s="8">
+        <v>976.45169999999996</v>
+      </c>
+      <c r="H1" s="8">
+        <v>999.59460000000001</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>49334</v>
+      </c>
+      <c r="B2" s="8">
+        <v>-30564.01171875</v>
+      </c>
+      <c r="C2" s="8">
+        <v>25469.041015625</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="8">
+        <v>453.59009990095001</v>
+      </c>
+      <c r="F2" s="8">
+        <v>1097.4834146476001</v>
+      </c>
+      <c r="G2" s="8">
+        <v>0</v>
+      </c>
+      <c r="H2" s="8">
+        <v>344.79668496229999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>49335</v>
+      </c>
+      <c r="B3" s="8">
+        <v>-30544.01171875</v>
+      </c>
+      <c r="C3" s="8">
+        <v>25469.041015625</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="8">
+        <v>221.09139411140001</v>
+      </c>
+      <c r="F3" s="8">
+        <v>867.41288168944004</v>
+      </c>
+      <c r="G3" s="8">
+        <v>141.62563744196001</v>
+      </c>
+      <c r="H3" s="8">
+        <v>208.73005418503999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>49336</v>
+      </c>
+      <c r="B4" s="8">
+        <v>-30524.01171875</v>
+      </c>
+      <c r="C4" s="8">
+        <v>25469.041015625</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="8">
+        <v>161.20219730375001</v>
+      </c>
+      <c r="F4" s="8">
+        <v>1053.0143533551</v>
+      </c>
+      <c r="G4" s="8">
+        <v>169.37373725923999</v>
+      </c>
+      <c r="H4" s="8">
+        <v>189.05971987928001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AD2889E-603A-4188-A56E-E8B1602F42FB}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="9">
+        <v>758.45190000000002</v>
+      </c>
+      <c r="F1" s="9">
+        <v>797.42639999999994</v>
+      </c>
+      <c r="G1" s="9">
+        <v>976.45169999999996</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="9">
+        <v>54690</v>
+      </c>
+      <c r="B2" s="9">
+        <v>-27061.76171875</v>
+      </c>
+      <c r="C2" s="9">
+        <v>23224.771484375</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="9">
+        <v>159.91791615919999</v>
+      </c>
+      <c r="F2" s="9">
+        <v>1098.6568525743</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="9">
+        <v>54691</v>
+      </c>
+      <c r="B3" s="9">
+        <v>-27041.76171875</v>
+      </c>
+      <c r="C3" s="9">
+        <v>23224.771484375</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="9">
+        <v>181.22691655762</v>
+      </c>
+      <c r="F3" s="9">
+        <v>1090.8025167487001</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="9">
+        <v>54692</v>
+      </c>
+      <c r="B4" s="9">
+        <v>-27021.76171875</v>
+      </c>
+      <c r="C4" s="9">
+        <v>23224.771484375</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="9">
+        <v>204.58876648117999</v>
+      </c>
+      <c r="F4" s="9">
+        <v>1759.2748306630999</v>
+      </c>
+      <c r="G4" s="9">
+        <v>647.70729296115996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>